<commit_message>
feat(residents): support localized import headers and persist new identity fields
Switch resident import templates to Chinese labels and localized values while keeping backward compatibility, and persist english_name/birth_date through migration plus edge write and validation flows.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/residents-import-template.xlsx
+++ b/public/residents-import-template.xlsx
@@ -413,73 +413,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>中文姓名</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>bedNumber</t>
+          <t>英文姓名</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>床號</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>區域</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>age</t>
+          <t>性別</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>admissionDate</t>
+          <t>出生日期</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>assessmentNextDueDate</t>
+          <t>年齡</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>fundingType</t>
+          <t>入院日期</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>serviceType</t>
+          <t>下次評估日期</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>dementiaLevel</t>
+          <t>資助類別</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>isSpecialCareCase</t>
+          <t>服務類型</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>healthCondition</t>
+          <t>認知障礙症程度</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>medicationRecord</t>
+          <t>是否Special Care Case</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>健康狀況</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>用藥記錄</t>
         </is>
       </c>
     </row>
@@ -491,56 +501,66 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Resident A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>T001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>A區</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>女</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1948-05-20</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>78</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>GradeA_Subsidized</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Subsidized_Rehab</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>甲一買位</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>資助復康服務</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>沒有認知障礙</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>步態訓練中</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>每日晚間服藥</t>
         </is>

</xml_diff>